<commit_message>
mexi em algumas coisas, mas seguimos olhando pra ver se n falta nada
</commit_message>
<xml_diff>
--- a/static/modelo_planilha.xlsx
+++ b/static/modelo_planilha.xlsx
@@ -1,104 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9d0867bf1a72efb/Documentos/Lab_LEP/static/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_0A1379904F778EE69A0FA3D873C6119571085A4A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BFF3104-C83E-45C2-A456-2647ADAF9589}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-192" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parametros" sheetId="1" r:id="rId1"/>
-    <sheet name="Materiais" sheetId="2" r:id="rId2"/>
-    <sheet name="Equipamentos" sheetId="3" r:id="rId3"/>
-    <sheet name="Experimentos" sheetId="4" r:id="rId4"/>
-    <sheet name="Alternativas" sheetId="5" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametros" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materiais" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipamentos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experimentos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alternativas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investimento" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FluxoCaixa" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
-  <si>
-    <t>nome</t>
-  </si>
-  <si>
-    <t>tempo</t>
-  </si>
-  <si>
-    <t>rendimento</t>
-  </si>
-  <si>
-    <t>energia</t>
-  </si>
-  <si>
-    <t>mao_obra</t>
-  </si>
-  <si>
-    <t>outros</t>
-  </si>
-  <si>
-    <t>quantidade_produzida</t>
-  </si>
-  <si>
-    <t>Projeto proposto</t>
-  </si>
-  <si>
-    <t>quantidade</t>
-  </si>
-  <si>
-    <t>preco</t>
-  </si>
-  <si>
-    <t>Reagente A</t>
-  </si>
-  <si>
-    <t>Reagente B</t>
-  </si>
-  <si>
-    <t>horas</t>
-  </si>
-  <si>
-    <t>custo_hora</t>
-  </si>
-  <si>
-    <t>Espectrofotômetro</t>
-  </si>
-  <si>
-    <t>Estufa</t>
-  </si>
-  <si>
-    <t>valor</t>
-  </si>
-  <si>
-    <t>custo</t>
-  </si>
-  <si>
-    <t>Método tradicional</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -117,21 +53,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -419,62 +414,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tempo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rendimento</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>mao_obra</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>outros</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>quantidade_produzida</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Projeto proposto</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
-        <v>6</v>
-      </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>15</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>150</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>800</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>100</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>50</v>
       </c>
     </row>
@@ -484,44 +490,54 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>quantidade</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>preco</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reagente A</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>10</v>
       </c>
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>25.5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Reagente B</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>5</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>40</v>
       </c>
     </row>
@@ -531,45 +547,54 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>horas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>custo_hora</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Espectrofotômetro</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Estufa</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2">
-        <v>8</v>
-      </c>
-      <c r="C2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
-        <v>12</v>
-      </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -579,35 +604,38 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>12.4</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" t="n">
         <v>12.7</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" t="n">
         <v>12.5</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" t="n">
         <v>12.6</v>
       </c>
     </row>
@@ -617,42 +645,148 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>custo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tempo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rendimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Método tradicional</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>investimento_inicial</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>taxa_desconto</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>valor_residual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>periodo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B2" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2">
-        <v>2200</v>
-      </c>
-      <c r="C2">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>10</v>
+      <c r="B3" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>